<commit_message>
feat: Agregar funcionalidad para generación de reportes de Plan de Viaje en formato Excel, incluyendo nuevos métodos y clases para manejo de viáticos y actualización de la interfaz de usuario
</commit_message>
<xml_diff>
--- a/src/WebApp.Web/Templates/PlanViajeTemplate.xlsx
+++ b/src/WebApp.Web/Templates/PlanViajeTemplate.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
   <si>
     <t>FONDO NACIONAL PARA LA REACTIVACIÓN Y MODERNIZACIÓN</t>
   </si>
@@ -98,9 +98,6 @@
     <t>Total  Q.</t>
   </si>
   <si>
-    <t>Totales</t>
-  </si>
-  <si>
     <t>TOTAL AUTORIZADO:</t>
   </si>
   <si>
@@ -122,15 +119,6 @@
     <t>Gerencia</t>
   </si>
   <si>
-    <t>{{Departamento}}</t>
-  </si>
-  <si>
-    <t>{{Fecha_Salida}}</t>
-  </si>
-  <si>
-    <t>{{Hora_Salida}}</t>
-  </si>
-  <si>
     <t>Fecha:</t>
   </si>
   <si>
@@ -140,25 +128,7 @@
     <t>Vo.Bo. Sub-Coordinador</t>
   </si>
   <si>
-    <t>{{Descripcion}}</t>
-  </si>
-  <si>
-    <t>{{fila_viatico}}</t>
-  </si>
-  <si>
-    <t>{{fila_destinos}}</t>
-  </si>
-  <si>
-    <t>{{Nombre}}</t>
-  </si>
-  <si>
-    <t>{{Monto_Aut}}</t>
-  </si>
-  <si>
-    <t>{{Fecha_Regreso}}</t>
-  </si>
-  <si>
-    <t>{{Hora_Regreso}}</t>
+    <t>||</t>
   </si>
 </sst>
 </file>
@@ -171,14 +141,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="&quot;Q&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -222,14 +185,17 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="12"/>
-      <name val="Arial"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -246,27 +212,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="7">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -279,88 +230,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -401,510 +275,130 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
-    <cellStyle name="Millares" xfId="1" builtinId="3"/>
-    <cellStyle name="Millares 2" xfId="3"/>
+  <cellStyles count="3">
+    <cellStyle name="Millares 2" xfId="2"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="16">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="d/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="d/m/yy"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="d/m/yy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="d/m/yy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="d/m/yy"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="double">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="double">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="double">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="double">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -978,37 +472,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Tabla25" displayName="Tabla25" ref="A22:E24" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13" headerRowCellStyle="Normal 2">
-  <autoFilter ref="A22:E24"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Descripción de Distancias" dataDxfId="12" dataCellStyle="Normal 2"/>
-    <tableColumn id="5" name="Kms." dataDxfId="11" dataCellStyle="Normal 2"/>
-    <tableColumn id="6" name="Galones" dataDxfId="10" dataCellStyle="Millares"/>
-    <tableColumn id="8" name="Precio Gal. Q" dataDxfId="9" dataCellStyle="Normal 2"/>
-    <tableColumn id="10" name="Total  Q." dataDxfId="8" dataCellStyle="Millares 2"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Tabla36" displayName="Tabla36" ref="A17:F19" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6" headerRowCellStyle="Normal 2" dataCellStyle="Millares 2">
-  <autoFilter ref="A17:F19"/>
-  <tableColumns count="6">
-    <tableColumn id="1" name="Fechas" dataDxfId="5" dataCellStyle="Normal 2"/>
-    <tableColumn id="2" name="Desayunos" dataDxfId="4" dataCellStyle="Millares 2"/>
-    <tableColumn id="3" name="Almuerzos" dataDxfId="3" dataCellStyle="Millares 2"/>
-    <tableColumn id="4" name="Cenas" dataDxfId="2" dataCellStyle="Millares 2"/>
-    <tableColumn id="5" name="Hospedaje" dataDxfId="1" dataCellStyle="Millares 2"/>
-    <tableColumn id="6" name="TOTAL" dataDxfId="0" dataCellStyle="Millares 2">
-      <calculatedColumnFormula>SUM(B18:E18)</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1274,14 +737,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:F47"/>
+  <dimension ref="A2:I47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="14.88671875" style="2" customWidth="1"/>
     <col min="3" max="3" width="12.109375" style="2" customWidth="1"/>
     <col min="4" max="4" width="11.21875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="13.77734375" style="2" customWidth="1"/>
     <col min="6" max="6" width="10.77734375" style="2" customWidth="1"/>
     <col min="7" max="240" width="11.5546875" style="2"/>
     <col min="241" max="241" width="7.88671875" style="2" customWidth="1"/>
@@ -1853,21 +1316,21 @@
     <col min="16124" max="16384" width="11.5546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" ht="12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="12" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:6" ht="12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="12" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="5" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="5"/>
       <c r="C5" s="6" t="s">
@@ -1876,7 +1339,7 @@
       <c r="D5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -1884,19 +1347,16 @@
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
     </row>
-    <row r="7" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A7" s="42" t="s">
+    <row r="7" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A7" s="23" t="s">
         <v>3</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
     </row>
-    <row r="8" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="5"/>
@@ -1904,49 +1364,41 @@
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
     </row>
-    <row r="9" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="53" t="s">
+    <row r="9" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="53"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="54" t="s">
+      <c r="B9" s="44"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="54"/>
-      <c r="F9" s="26"/>
-    </row>
-    <row r="10" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A10" s="35" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" s="33" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="33"/>
-      <c r="D10" s="35" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="33" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="34"/>
-      <c r="D11" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="34" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E9" s="45"/>
+      <c r="F9" s="15"/>
+    </row>
+    <row r="10" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A10" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="20"/>
+    </row>
+    <row r="11" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="21"/>
+    </row>
+    <row r="12" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="5"/>
@@ -1954,8 +1406,8 @@
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:6" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="44" t="s">
+    <row r="13" spans="1:9" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="25" t="s">
         <v>6</v>
       </c>
       <c r="B13" s="5"/>
@@ -1964,25 +1416,26 @@
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
     </row>
-    <row r="14" spans="1:6" ht="68.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="55" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="56"/>
-      <c r="C14" s="56"/>
-      <c r="D14" s="56"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="57"/>
-    </row>
-    <row r="15" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A15" s="49"/>
-      <c r="B15" s="50"/>
-      <c r="C15" s="50"/>
-      <c r="D15" s="50"/>
-      <c r="E15" s="50"/>
+    <row r="14" spans="1:9" ht="68.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="46"/>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="48"/>
+      <c r="I14" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A15" s="30"/>
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
       <c r="F15" s="5"/>
     </row>
-    <row r="16" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>7</v>
       </c>
@@ -1992,58 +1445,51 @@
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
     </row>
-    <row r="17" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A17" s="37" t="s">
+    <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A17" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="38" t="s">
+      <c r="B17" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="38" t="s">
+      <c r="C17" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="38" t="s">
+      <c r="D17" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="E17" s="38" t="s">
+      <c r="E17" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="F17" s="39" t="s">
+      <c r="F17" s="40" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="41" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="40"/>
-    </row>
-    <row r="19" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="18" t="s">
+    <row r="18" spans="1:6" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="41"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="42"/>
+    </row>
+    <row r="19" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="21">
-        <f>SUM(B18:B18)</f>
+      <c r="B19" s="42">
         <v>0</v>
       </c>
-      <c r="C19" s="21">
-        <f>SUM(C18:C18)</f>
+      <c r="C19" s="42">
         <v>0</v>
       </c>
-      <c r="D19" s="21">
-        <f>SUM(D18:D18)</f>
+      <c r="D19" s="42">
         <v>0</v>
       </c>
-      <c r="E19" s="21">
-        <f>SUM(E18:E18)</f>
+      <c r="E19" s="42">
         <v>0</v>
       </c>
-      <c r="F19" s="21">
-        <f>SUM(B19:E19)</f>
+      <c r="F19" s="42">
         <v>0</v>
       </c>
     </row>
@@ -2067,81 +1513,73 @@
       <c r="E21" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F21" s="30"/>
-    </row>
-    <row r="22" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
+      <c r="F21" s="19"/>
+    </row>
+    <row r="22" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="D22" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="F22" s="32"/>
-    </row>
-    <row r="23" spans="1:6" ht="12.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="31"/>
-    </row>
-    <row r="24" spans="1:6" ht="12.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" s="19">
-        <f>SUM(B23:B23)</f>
+      <c r="F22"/>
+    </row>
+    <row r="23" spans="1:6" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="34"/>
+      <c r="B23"/>
+      <c r="C23" s="36"/>
+      <c r="D23"/>
+      <c r="E23" s="35"/>
+      <c r="F23"/>
+    </row>
+    <row r="24" spans="1:6" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="37" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="35">
         <v>0</v>
       </c>
-      <c r="C24" s="20">
-        <f>SUM(C23:C23)</f>
+      <c r="C24" s="36">
         <v>0</v>
       </c>
-      <c r="D24" s="19">
-        <f>D23</f>
+      <c r="D24" s="35">
         <v>0</v>
       </c>
-      <c r="E24" s="21">
-        <f>SUM(E23:F23)</f>
+      <c r="E24" s="35">
         <v>0</v>
       </c>
-      <c r="F24" s="30"/>
+      <c r="F24"/>
     </row>
     <row r="25" spans="1:6" ht="12.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="30"/>
+      <c r="A25" s="11"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="19"/>
     </row>
     <row r="26" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
-      <c r="E26" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="F26" s="51" t="s">
-        <v>41</v>
-      </c>
+      <c r="E26" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26" s="32"/>
     </row>
     <row r="27" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -2166,19 +1604,17 @@
       <c r="F29" s="8"/>
     </row>
     <row r="30" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A30" s="47" t="s">
-        <v>40</v>
-      </c>
-      <c r="C30" s="43"/>
+      <c r="A30" s="28"/>
+      <c r="C30" s="24"/>
       <c r="D30" s="8"/>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A31" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="C31" s="25"/>
+      <c r="A31" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="14"/>
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
@@ -2200,38 +1636,38 @@
       <c r="F33" s="5"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="28"/>
+      <c r="A35" s="17"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A36" s="45" t="s">
+      <c r="A36" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="D36" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C38" s="16"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46" s="13"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="D36" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="E36" s="28"/>
-      <c r="F36" s="28"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C38" s="27"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A46" s="14"/>
-      <c r="C46" s="27"/>
-      <c r="D46" s="46" t="s">
+      <c r="E46" s="17"/>
+      <c r="F46" s="17"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="E47" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="E46" s="28"/>
-      <c r="F46" s="28"/>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A47" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="E47" s="52" t="s">
-        <v>30</v>
-      </c>
-      <c r="F47" s="29"/>
+      <c r="F47" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2247,9 +1683,5 @@
     <brk id="6" max="1048575" man="1"/>
   </colBreaks>
   <drawing r:id="rId2"/>
-  <tableParts count="2">
-    <tablePart r:id="rId3"/>
-    <tablePart r:id="rId4"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: YA FUNCIONA EL CREAR PLAN DE VIAJES Y  Agregar detalles de destinos en Plan de Viaje, incluyendo cálculos de combustible y actualización de la interfaz de usuario
</commit_message>
<xml_diff>
--- a/src/WebApp.Web/Templates/PlanViajeTemplate.xlsx
+++ b/src/WebApp.Web/Templates/PlanViajeTemplate.xlsx
@@ -14,9 +14,6 @@
   <sheets>
     <sheet name="PlanViajeTemplate" sheetId="3" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">PlanViajeTemplate!#REF!</definedName>
-  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -128,7 +125,7 @@
     <t>Vo.Bo. Sub-Coordinador</t>
   </si>
   <si>
-    <t>||</t>
+    <t>Quetzaltenango</t>
   </si>
 </sst>
 </file>
@@ -212,7 +209,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -290,13 +287,151 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -361,22 +496,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -391,6 +515,43 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -737,10 +898,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:I47"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:F47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="34.109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="31.88671875" style="1" customWidth="1"/>
     <col min="2" max="2" width="14.88671875" style="2" customWidth="1"/>
     <col min="3" max="3" width="12.109375" style="2" customWidth="1"/>
     <col min="4" max="4" width="11.21875" style="2" customWidth="1"/>
@@ -1316,21 +1480,21 @@
     <col min="16124" max="16384" width="11.5546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" ht="12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="12" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:9" ht="12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="12" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="5" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="5"/>
       <c r="C5" s="6" t="s">
@@ -1339,7 +1503,7 @@
       <c r="D5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -1347,16 +1511,19 @@
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
     </row>
-    <row r="7" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
         <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>33</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
     </row>
-    <row r="8" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="5"/>
@@ -1364,41 +1531,41 @@
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
     </row>
-    <row r="9" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="44" t="s">
+    <row r="9" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="44"/>
+      <c r="B9" s="37"/>
       <c r="C9" s="14"/>
-      <c r="D9" s="45" t="s">
+      <c r="D9" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="45"/>
+      <c r="E9" s="38"/>
       <c r="F9" s="15"/>
     </row>
-    <row r="10" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="20"/>
+      <c r="B10" s="57"/>
       <c r="C10" s="20"/>
       <c r="D10" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="20"/>
-    </row>
-    <row r="11" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E10" s="57"/>
+    </row>
+    <row r="11" spans="1:6" ht="13.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="21"/>
+      <c r="B11" s="58"/>
       <c r="C11" s="21"/>
       <c r="D11" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E11" s="21"/>
-    </row>
-    <row r="12" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E11" s="58"/>
+    </row>
+    <row r="12" spans="1:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="5"/>
@@ -1406,7 +1573,7 @@
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:9" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="25" t="s">
         <v>6</v>
       </c>
@@ -1416,18 +1583,15 @@
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
     </row>
-    <row r="14" spans="1:9" ht="68.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="46"/>
-      <c r="B14" s="47"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="48"/>
-      <c r="I14" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="68.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="39"/>
+      <c r="B14" s="40"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="41"/>
+    </row>
+    <row r="15" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="30"/>
       <c r="B15" s="31"/>
       <c r="C15" s="31"/>
@@ -1435,61 +1599,71 @@
       <c r="E15" s="31"/>
       <c r="F15" s="5"/>
     </row>
-    <row r="16" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+    <row r="16" spans="1:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="47"/>
     </row>
     <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="40" t="s">
+      <c r="B17" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="40" t="s">
+      <c r="C17" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="40" t="s">
+      <c r="D17" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="E17" s="40" t="s">
+      <c r="E17" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="F17" s="40" t="s">
+      <c r="F17" s="56" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="41"/>
-      <c r="B18" s="42"/>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="42"/>
-    </row>
-    <row r="19" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="43" t="s">
+      <c r="A18" s="49"/>
+      <c r="B18" s="34">
+        <v>0</v>
+      </c>
+      <c r="C18" s="34">
+        <v>0</v>
+      </c>
+      <c r="D18" s="34">
+        <v>0</v>
+      </c>
+      <c r="E18" s="34">
+        <v>0</v>
+      </c>
+      <c r="F18" s="44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="42">
+      <c r="B19" s="43">
         <v>0</v>
       </c>
-      <c r="C19" s="42">
+      <c r="C19" s="43">
         <v>0</v>
       </c>
-      <c r="D19" s="42">
+      <c r="D19" s="43">
         <v>0</v>
       </c>
-      <c r="E19" s="42">
+      <c r="E19" s="43">
         <v>0</v>
       </c>
-      <c r="F19" s="42">
+      <c r="F19" s="45">
         <v>0</v>
       </c>
     </row>
@@ -1501,7 +1675,7 @@
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
     </row>
-    <row r="21" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>15</v>
       </c>
@@ -1516,45 +1690,53 @@
       <c r="F21" s="19"/>
     </row>
     <row r="22" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="38" t="s">
+      <c r="A22" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="39" t="s">
+      <c r="B22" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="39" t="s">
+      <c r="C22" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="39" t="s">
+      <c r="D22" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="E22" s="39" t="s">
+      <c r="E22" s="52" t="s">
         <v>22</v>
       </c>
       <c r="F22"/>
     </row>
     <row r="23" spans="1:6" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="34"/>
-      <c r="B23"/>
-      <c r="C23" s="36"/>
-      <c r="D23"/>
-      <c r="E23" s="35"/>
+      <c r="A23" s="53"/>
+      <c r="B23" s="34">
+        <v>0</v>
+      </c>
+      <c r="C23" s="35">
+        <v>0</v>
+      </c>
+      <c r="D23" s="34">
+        <v>0</v>
+      </c>
+      <c r="E23" s="44">
+        <v>0</v>
+      </c>
       <c r="F23"/>
     </row>
-    <row r="24" spans="1:6" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="37" t="s">
+    <row r="24" spans="1:6" ht="12.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="35">
+      <c r="B24" s="43">
         <v>0</v>
       </c>
-      <c r="C24" s="36">
+      <c r="C24" s="54">
         <v>0</v>
       </c>
-      <c r="D24" s="35">
+      <c r="D24" s="43">
         <v>0</v>
       </c>
-      <c r="E24" s="35">
+      <c r="E24" s="45">
         <v>0</v>
       </c>
       <c r="F24"/>
@@ -1567,12 +1749,12 @@
       <c r="E25" s="12"/>
       <c r="F25" s="19"/>
     </row>
-    <row r="26" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
-      <c r="E26" s="12" t="s">
+      <c r="E26" s="36" t="s">
         <v>23</v>
       </c>
       <c r="F26" s="32"/>
@@ -1585,7 +1767,7 @@
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
+      <c r="F27" s="42"/>
     </row>
     <row r="28" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
@@ -1619,7 +1801,7 @@
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
       <c r="B32" s="8"/>
       <c r="C32" s="5"/>
@@ -1677,7 +1859,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.9055118110236221" bottom="0.39370078740157483" header="0" footer="0"/>
-  <pageSetup scale="76" orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="6" max="1048575" man="1"/>

</xml_diff>